<commit_message>
chore: record Udyam UDYAM-KR-03-0774393 as completed (15 Oct 2026)
Update STATUS.md business launch section (Udyam Completed; GST Completed
14 Oct) and sync Launch Checklist tracker into common/.
</commit_message>
<xml_diff>
--- a/common/SPICO_Vita_Tracker.xlsx
+++ b/common/SPICO_Vita_Tracker.xlsx
@@ -616,7 +616,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -629,6 +629,11 @@
       </c>
       <c r="H5" s="3" t="n">
         <v>46310</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>UDYAM-KR-03-0774393 registered 15 Oct 2026 (free at udyamregistration.gov.in)</t>
+        </is>
       </c>
     </row>
     <row r="6">

</xml_diff>